<commit_message>
v2.3.0: Sector-company-v2 (135 stocks), dynamic count, Trending 50% Z(RSI)+50% Z(CMF), df_stocks fix, CHANGES_LOG/CHANGES_SUMMARY
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Sector-Company.xlsx
+++ b/Sector-Company.xlsx
@@ -633,197 +633,179 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Commodities</t>
+          <t>Auto</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Hindalco Industries</t>
+          <t>M&amp;M</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>HINDALCO.NS</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>25.3</v>
-      </c>
+          <t>M&amp;M.NS</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Commodities</t>
+          <t>Auto</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>NMDC Limited</t>
+          <t>Tata Motors Passenger Vehicles</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>NMDC.NS</t>
-        </is>
-      </c>
-      <c r="D12" t="n">
-        <v>18.7</v>
-      </c>
+          <t>TMPV.NS</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Commodities</t>
+          <t>Auto</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Coal India</t>
+          <t>TVS Motor</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>COALINDIA.NS</t>
-        </is>
-      </c>
-      <c r="D13" t="n">
-        <v>15.2</v>
-      </c>
+          <t>TVSMOTOR.NS</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Commodities</t>
+          <t>Auto</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Fineotex Chemical</t>
+          <t>Motherson Sumi Systems</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>FINEOTEX.NS</t>
-        </is>
-      </c>
-      <c r="D14" t="n">
-        <v>12.1</v>
-      </c>
+          <t>MOTHERSON.NS</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Commodities</t>
+          <t>Auto</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Ratnamani Metals</t>
+          <t>Timken India</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>RATNAMANI.NS</t>
-        </is>
-      </c>
-      <c r="D15" t="n">
-        <v>8.9</v>
-      </c>
+          <t>TIINDIA.NS</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Commodities</t>
+          <t>Auto</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Jindal Steel</t>
+          <t>MRF Limited</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>JINDALSTEL.NS</t>
-        </is>
-      </c>
-      <c r="D16" t="n">
-        <v>7.8</v>
-      </c>
+          <t>MRF.NS</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Commodities</t>
+          <t>Auto</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Vedanta</t>
+          <t>Apollo Tyres</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>VEDL.NS</t>
-        </is>
-      </c>
-      <c r="D17" t="n">
-        <v>6.4</v>
-      </c>
+          <t>APOLLOTYRE.NS</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Commodities</t>
+          <t>Auto</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Manganese Ore India</t>
+          <t>Exide Industries</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>MOIL.NS</t>
-        </is>
-      </c>
-      <c r="D18" t="n">
-        <v>5.6</v>
-      </c>
+          <t>EXIDEIND.NS</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Defence</t>
+          <t>Auto</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Bharat Electronics</t>
+          <t>Balkrishna Industries</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>BEL.NS</t>
-        </is>
-      </c>
-      <c r="D19" t="n">
-        <v>28.5</v>
-      </c>
+          <t>BALKRISIND.NS</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Defence</t>
+          <t>Commodities</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Hindustan Aeronautics</t>
+          <t>Hindalco Industries</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>HAL.NS</t>
+          <t>HINDALCO.NS</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -833,17 +815,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Defence</t>
+          <t>Commodities</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Mazagon Dock</t>
+          <t>NMDC Limited</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>MAZDOCK.NS</t>
+          <t>NMDC.NS</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -853,1557 +835,1505 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Defence</t>
+          <t>Commodities</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Bharat Dynamics</t>
+          <t>Coal India</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>BDL.NS</t>
+          <t>COALINDIA.NS</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>5.2</v>
+        <v>15.2</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Commodities</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Reliance Industries</t>
+          <t>Fineotex Chemical</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>RELIANCE.NS</t>
+          <t>FINEOTEX.NS</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>35.2</v>
+        <v>12.1</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Commodities</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>NTPC Limited</t>
+          <t>Ratnamani Metals</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>NTPC.NS</t>
+          <t>RATNAMANI.NS</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>18.9</v>
+        <v>8.9</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Commodities</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Power Grid</t>
+          <t>Jindal Steel</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>POWERGRID.NS</t>
+          <t>JINDALSTEL.NS</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>12.3</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Fin Services</t>
+          <t>Commodities</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Bajaj Finance Ltd.</t>
+          <t>Manganese Ore India</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>BAJFINANCE.NS</t>
+          <t>MOIL.NS</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>15.4</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Fin Services</t>
+          <t>Commodities</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Shriram Finance Ltd.</t>
+          <t>Vedanta</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>SHRIRAMFIN.NS</t>
+          <t>VEDL.NS</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>8.199999999999999</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Fin Services</t>
+          <t>Consumer Durable</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Bajaj Finserv Ltd.</t>
+          <t>Titan Company</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>BAJAJFINSV.NS</t>
-        </is>
-      </c>
-      <c r="D28" t="n">
-        <v>6.85</v>
-      </c>
+          <t>TITAN.NS</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Fin Services</t>
+          <t>Consumer Durable</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>BSE Ltd.</t>
+          <t>Dixon Technologies</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>BSE.NS</t>
-        </is>
-      </c>
-      <c r="D29" t="n">
-        <v>6.32</v>
-      </c>
+          <t>DIXON.NS</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Fin Services</t>
+          <t>Consumer Durable</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Jio Financial Services Ltd.</t>
+          <t>Havells India</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>JIOFIN.NS</t>
-        </is>
-      </c>
-      <c r="D30" t="n">
-        <v>5.68</v>
-      </c>
+          <t>HAVELLS.NS</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Fin Services</t>
+          <t>Consumer Durable</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>SBI Life Insurance Company</t>
+          <t>Voltas</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>SBILIFE.NS</t>
-        </is>
-      </c>
-      <c r="D31" t="n">
-        <v>5.37</v>
-      </c>
+          <t>VOLTAS.NS</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Fin Services</t>
+          <t>Consumer Durable</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>HDFC Life Insurance Company</t>
+          <t>Blue Star</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>HDFCLIFE.NS</t>
-        </is>
-      </c>
-      <c r="D32" t="n">
-        <v>4.74</v>
-      </c>
+          <t>BLUESTARCO.NS</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Fin Services</t>
+          <t>Consumer Durable</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Cholamandalam Inv. &amp; Fin.</t>
+          <t>Kajaria Ceramics</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>CHOLAFIN.NS</t>
-        </is>
-      </c>
-      <c r="D33" t="n">
-        <v>4.23</v>
-      </c>
+          <t>KAJARIACER.NS</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Fin Services</t>
+          <t>Consumer Durable</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>PB Fintech (Policybazaar)</t>
+          <t>Thangamayil Jewellery</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>POLICYBZR.NS</t>
-        </is>
-      </c>
-      <c r="D34" t="n">
-        <v>3.66</v>
-      </c>
+          <t>THANGAMAYL.NS</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Fin Services</t>
+          <t>Consumer Durable</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>MCX India Ltd.</t>
+          <t>PNG Jewellers</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>MCX.NS</t>
-        </is>
-      </c>
-      <c r="D35" t="n">
-        <v>3.34</v>
-      </c>
+          <t>PNGJL.NS</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Fin Services</t>
+          <t>Consumer Durable</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>PNB Housing</t>
+          <t>Kalyan Jewellers India</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>PNBHOUSING.NS</t>
-        </is>
-      </c>
-      <c r="D36" t="n">
-        <v>1.9</v>
-      </c>
+          <t>KALYANKJIL.NS</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Fin Services</t>
+          <t>Defence</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>HDFC Asset Management</t>
+          <t>Bharat Electronics</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>HDFCAMC.NS</t>
+          <t>BEL.NS</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>1.3</v>
+        <v>28.5</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Fin Services</t>
+          <t>Defence</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Manappuram Finance</t>
+          <t>Hindustan Aeronautics</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>MANAPPURAM.NS</t>
+          <t>HAL.NS</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>1</v>
+        <v>25.3</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>FMCG</t>
+          <t>Defence</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>ITC Limited</t>
+          <t>Mazagon Dock</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>ITC.NS</t>
+          <t>MAZDOCK.NS</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>22.3</v>
+        <v>18.7</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>FMCG</t>
+          <t>Defence</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Nestle India</t>
+          <t>Bharat Dynamics</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>NESTLEIND.NS</t>
+          <t>BDL.NS</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>18.9</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>FMCG</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Hindustan Unilever</t>
+          <t>Reliance Industries</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>HINDUNILVR.NS</t>
+          <t>RELIANCE.NS</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>17.5</v>
+        <v>35.2</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>FMCG</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Marico</t>
+          <t>NTPC Limited</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>MARICO.NS</t>
+          <t>NTPC.NS</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>12.1</v>
+        <v>18.9</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>FMCG</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Britannia Industries</t>
+          <t>Power Grid Corporation</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>BRITANNIA.NS</t>
+          <t>POWERGRID.NS</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>10.8</v>
+        <v>12.3</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>FMCG</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Godrej Industries</t>
+          <t>Tata Power</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>GODREJIND.NS</t>
-        </is>
-      </c>
-      <c r="D44" t="n">
-        <v>8.199999999999999</v>
-      </c>
+          <t>TATAPOWER.NS</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>FMCG</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Emami Limited</t>
+          <t>Adani Green Energy</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>EMAMILTD.NS</t>
-        </is>
-      </c>
-      <c r="D45" t="n">
-        <v>5.6</v>
-      </c>
+          <t>ADANIGREEN.NS</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>FMCG</t>
+          <t>Fin Services</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Colgate-Palmolive</t>
+          <t>Bajaj Finance Ltd.</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>COLPAL.NS</t>
+          <t>BAJFINANCE.NS</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>4.6</v>
+        <v>15.4</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Infra</t>
+          <t>Fin Services</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Larsen &amp; Toubro</t>
+          <t>Shriram Finance Ltd.</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>LT.NS</t>
+          <t>SHRIRAMFIN.NS</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>24.3</v>
+        <v>8.199999999999999</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Infra</t>
+          <t>Fin Services</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Indian Railway Finance</t>
+          <t>Bajaj Finserv Ltd.</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>IRFC.NS</t>
+          <t>BAJAJFINSV.NS</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>15.8</v>
+        <v>6.85</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Infra</t>
+          <t>Fin Services</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>NHPC Limited</t>
+          <t>BSE Ltd.</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>NHPC.NS</t>
+          <t>BSE.NS</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>12.5</v>
+        <v>6.32</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Infra</t>
+          <t>Fin Services</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Bharat Petroleum</t>
+          <t>Jio Financial Services Ltd.</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>BPCL.NS</t>
+          <t>JIOFIN.NS</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>9.699999999999999</v>
+        <v>5.68</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Infra</t>
+          <t>Fin Services</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>REC Limited</t>
+          <t>SBI Life Insurance Company</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>REC.NS</t>
+          <t>SBILIFE.NS</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>6.4</v>
+        <v>5.37</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Fin Services</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Tata Consultancy Services</t>
+          <t>HDFC Life Insurance Company</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>TCS.NS</t>
+          <t>HDFCLIFE.NS</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>20.5</v>
+        <v>4.74</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Fin Services</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Infosys</t>
+          <t>Cholamandalam Inv. &amp; Fin.</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>INFY.NS</t>
+          <t>CHOLAFIN.NS</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>18.2</v>
+        <v>4.23</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Fin Services</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Wipro</t>
+          <t>PB Fintech (Policybazaar)</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>WIPRO.NS</t>
+          <t>POLICYBZR.NS</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>12.1</v>
+        <v>3.66</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Fin Services</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Tech Mahindra</t>
+          <t>MCX India Ltd.</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>TECHM.NS</t>
+          <t>MCX.NS</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>9.800000000000001</v>
+        <v>3.34</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Fin Services</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>HCL Technologies</t>
+          <t>PNB Housing Finance</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>HCLTECH.NS</t>
+          <t>PNBHOUSING.NS</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>7.3</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Fin Services</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Persistent</t>
+          <t>HDFC Asset Management</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>PERSISTENT.NS</t>
+          <t>HDFCAMC.NS</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>6.4</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Fin Services</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Coforge</t>
+          <t>Manappuram Finance</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>COFORGE.NS</t>
+          <t>MANAPPURAM.NS</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>5.3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Fin Services</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Mphasis</t>
+          <t>LT Finance</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>MPHASIS.NS</t>
-        </is>
-      </c>
-      <c r="D59" t="n">
-        <v>5.2</v>
-      </c>
+          <t>LTF.NS</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Fin Services</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>LT Technologies</t>
+          <t>Muthoot Finance</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>LTTS.NS</t>
-        </is>
-      </c>
-      <c r="D60" t="n">
-        <v>4.1</v>
-      </c>
+          <t>MUTHOOTFIN.NS</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Fin Services</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Sun TV Network</t>
+          <t>AB Capital</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>SUNTV.NS</t>
-        </is>
-      </c>
-      <c r="D61" t="n">
-        <v>18.5</v>
-      </c>
+          <t>ABCAPITAL.NS</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>FMCG</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Zee Entertainment</t>
+          <t>ITC Limited</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>ZEEL.NS</t>
+          <t>ITC.NS</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>12.8</v>
+        <v>22.3</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>FMCG</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>TV Today</t>
+          <t>Nestle India</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>TVTODAY.NS</t>
+          <t>NESTLEIND.NS</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>10.2</v>
+        <v>18.9</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>FMCG</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Network 18</t>
+          <t>Hindustan Unilever</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>NETWORK18.NS</t>
+          <t>HINDUNILVR.NS</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>8.9</v>
+        <v>17.5</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Metal</t>
+          <t>FMCG</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Tata Steel</t>
+          <t>Marico</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>TATASTEEL.NS</t>
+          <t>MARICO.NS</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>27.7</v>
+        <v>12.1</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Metal</t>
+          <t>FMCG</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>JSW Steel</t>
+          <t>Britannia Industries</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>JSWSTEEL.NS</t>
+          <t>BRITANNIA.NS</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>17.9</v>
+        <v>10.8</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Metal</t>
+          <t>FMCG</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>National Aluminium</t>
+          <t>Godrej Industries</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>NATIONALUM.NS</t>
+          <t>GODREJIND.NS</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>5.7</v>
+        <v>8.199999999999999</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Nifty 50</t>
+          <t>FMCG</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>HDFC Bank</t>
+          <t>Emami Limited</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>HDFCBANK.NS</t>
+          <t>EMAMILTD.NS</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>8.199999999999999</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Nifty 50</t>
+          <t>FMCG</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>ICICI Bank</t>
+          <t>Colgate-Palmolive</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>ICICIBANK.NS</t>
+          <t>COLPAL.NS</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>6.3</v>
+        <v>4.6</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Nifty 50</t>
+          <t>FMCG</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>State Bank of India</t>
+          <t>Dabur India</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>SBIN.NS</t>
-        </is>
-      </c>
-      <c r="D70" t="n">
-        <v>5.1</v>
-      </c>
+          <t>DABUR.NS</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Oil &amp; Gas</t>
+          <t>FMCG</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Indian Oil Corporation</t>
+          <t>Varun Beverages</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>IOC.NS</t>
-        </is>
-      </c>
-      <c r="D71" t="n">
-        <v>18.5</v>
-      </c>
+          <t>VBL.NS</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Oil &amp; Gas</t>
+          <t>FMCG</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Oil and Natural Gas</t>
+          <t>Godrej Consumer Products</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>ONGC.NS</t>
-        </is>
-      </c>
-      <c r="D72" t="n">
-        <v>10.2</v>
-      </c>
+          <t>GODREJCP.NS</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Oil &amp; Gas</t>
+          <t>FMCG</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Gas Authority of India</t>
+          <t>Tata Consumer Products</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>GAIL.NS</t>
-        </is>
-      </c>
-      <c r="D73" t="n">
-        <v>3.8</v>
-      </c>
+          <t>TATACONSUM.NS</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Pharma</t>
+          <t>Infra</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Sun Pharmaceutical</t>
+          <t>Larsen &amp; Toubro</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>SUNPHARMA.NS</t>
+          <t>LT.NS</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>18.5</v>
+        <v>24.3</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Pharma</t>
+          <t>Infra</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Lupin Limited</t>
+          <t>Indian Railway Finance</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>LUPIN.NS</t>
+          <t>IRFC.NS</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>14.2</v>
+        <v>15.8</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Pharma</t>
+          <t>Infra</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Cipla</t>
+          <t>NHPC Limited</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>CIPLA.NS</t>
+          <t>NHPC.NS</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>12.8</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Pharma</t>
+          <t>Infra</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Dr. Reddy's Labs</t>
+          <t>REC Limited</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>DRREDDY.NS</t>
+          <t>REC.NS</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>11.5</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Pharma</t>
+          <t>Infra</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Aurobindo Pharma</t>
+          <t>Bharti Airtel</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>AUROPHARMA.NS</t>
-        </is>
-      </c>
-      <c r="D78" t="n">
-        <v>9.699999999999999</v>
-      </c>
+          <t>BHARTIARTL.NS</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Pharma</t>
+          <t>Infra</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Divi's Laboratories</t>
+          <t>Adani Ports &amp; SEZ</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>DIVISLAB.NS</t>
-        </is>
-      </c>
-      <c r="D79" t="n">
-        <v>8.300000000000001</v>
-      </c>
+          <t>ADANIPORTS.NS</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Pharma</t>
+          <t>Infra</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>IPCA Laboratories</t>
+          <t>IndiGo</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>IPCALAB.NS</t>
-        </is>
-      </c>
-      <c r="D80" t="n">
-        <v>6.9</v>
-      </c>
+          <t>INDIGO.NS</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Pharma</t>
+          <t>Infra</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Alembic Pharma</t>
+          <t>Grasim Industries</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>APLLTD.NS</t>
-        </is>
-      </c>
-      <c r="D81" t="n">
-        <v>5.8</v>
-      </c>
+          <t>GRASIM.NS</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>PSU Bank</t>
+          <t>Infra</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Central Bank</t>
+          <t>JSW Energy</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>CENTRALBK.NS</t>
-        </is>
-      </c>
-      <c r="D82" t="n">
-        <v>18.5</v>
-      </c>
+          <t>JSWENERGY.NS</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>PSU Bank</t>
+          <t>Infra</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Bank of Baroda</t>
+          <t>Siemens Limited</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>BANKBARODA.NS</t>
-        </is>
-      </c>
-      <c r="D83" t="n">
-        <v>15.3</v>
-      </c>
+          <t>SIEMENS.NS</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>PSU Bank</t>
+          <t>Infra</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Indian Bank</t>
+          <t>Cummins India</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>INDIANB.NS</t>
-        </is>
-      </c>
-      <c r="D84" t="n">
-        <v>12.1</v>
-      </c>
+          <t>CUMMINSIND.NS</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>PSU Bank</t>
+          <t>Infra</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Canara Bank</t>
+          <t>Shree Cement</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>CANBK.NS</t>
-        </is>
-      </c>
-      <c r="D85" t="n">
-        <v>9.800000000000001</v>
-      </c>
+          <t>SHREECEM.NS</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>PSU Bank</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Union Bank</t>
+          <t>Tata Consultancy Services</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>UNIONBANK.NS</t>
+          <t>TCS.NS</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>4.2</v>
+        <v>20.5</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Pvt Bank</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Axis Bank</t>
+          <t>Infosys</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>AXISBANK.NS</t>
+          <t>INFY.NS</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>18.7</v>
+        <v>18.2</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Pvt Bank</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Kotak Mahindra Bank</t>
+          <t>Wipro</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>KOTAKBANK.NS</t>
+          <t>WIPRO.NS</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>15.2</v>
+        <v>12.1</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Pvt Bank</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>IDFC First Bank</t>
+          <t>Tech Mahindra</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>IDFCFIRSTB.NS</t>
+          <t>TECHM.NS</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>7.8</v>
+        <v>9.800000000000001</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Pvt Bank</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>IndusInd Bank</t>
+          <t>HCL Technologies</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>INDUSINDBK.NS</t>
+          <t>HCLTECH.NS</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>4.2</v>
+        <v>7.3</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Realty</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>DLF Limited</t>
+          <t>Persistent Systems</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>DLF.NS</t>
+          <t>PERSISTENT.NS</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>22.5</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Realty</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Sunteck Realty</t>
+          <t>Coforge</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>SUNTECK.NS</t>
+          <t>COFORGE.NS</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>18.3</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Realty</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Oberoi Realty</t>
+          <t>Mphasis</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>OBEROIRLTY.NS</t>
+          <t>MPHASIS.NS</t>
         </is>
       </c>
       <c r="D93" t="n">
-        <v>14</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Realty</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Prestige Estates</t>
+          <t>LT Technologies</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>PRESTIGE.NS</t>
+          <t>LTTS.NS</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>11.8</v>
+        <v>4.1</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Realty</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Lodha Group</t>
+          <t>Sun TV Network</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>LODHA.NS</t>
+          <t>SUNTV.NS</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>10.2</v>
+        <v>18.5</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Realty</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Indiabulls Real Estate</t>
+          <t>Zee Entertainment</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>IBREALEST.NS</t>
+          <t>ZEEL.NS</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>8.6</v>
+        <v>12.8</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Realty</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Brigade Enterprises</t>
+          <t>TV Today</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>BRIGADE.NS</t>
+          <t>TVTODAY.NS</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>8</v>
+        <v>10.2</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Realty</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Godrej Properties</t>
+          <t>Network 18</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>GODREJPROP.NS</t>
+          <t>NETWORK18.NS</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>6.7</v>
+        <v>8.9</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Auto</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Samvardhana Motherson</t>
+          <t>PVR INOX</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>MOTHERSON.NS</t>
+          <t>PVRINOX.NS</t>
         </is>
       </c>
       <c r="D99" t="inlineStr"/>
@@ -2411,272 +2341,302 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Auto</t>
+          <t>Metal</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Minda Corporation</t>
+          <t>Tata Steel</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>MINDACORP.NS</t>
-        </is>
-      </c>
-      <c r="D100" t="inlineStr"/>
+          <t>TATASTEEL.NS</t>
+        </is>
+      </c>
+      <c r="D100" t="n">
+        <v>27.7</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Commodities</t>
+          <t>Metal</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>SAIL</t>
+          <t>JSW Steel</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>SAIL.NS</t>
-        </is>
-      </c>
-      <c r="D101" t="inlineStr"/>
+          <t>JSWSTEEL.NS</t>
+        </is>
+      </c>
+      <c r="D101" t="n">
+        <v>17.9</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Defence</t>
+          <t>Metal</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Paras Defence</t>
+          <t>National Aluminium</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>PARAS.NS</t>
-        </is>
-      </c>
-      <c r="D102" t="inlineStr"/>
+          <t>NATIONALUM.NS</t>
+        </is>
+      </c>
+      <c r="D102" t="n">
+        <v>5.7</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Oil &amp; Gas</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Tata Power</t>
+          <t>Bharat Petroleum</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>TATAPOWER.NS</t>
-        </is>
-      </c>
-      <c r="D103" t="inlineStr"/>
+          <t>BPCL.NS</t>
+        </is>
+      </c>
+      <c r="D103" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Oil &amp; Gas</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Adani Green Energy</t>
+          <t>Indian Oil Corporation</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>ADANIGREEN.NS</t>
-        </is>
-      </c>
-      <c r="D104" t="inlineStr"/>
+          <t>IOC.NS</t>
+        </is>
+      </c>
+      <c r="D104" t="n">
+        <v>18.5</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Fin Services</t>
+          <t>Oil &amp; Gas</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>ICICI Lombard</t>
+          <t>Oil and Natural Gas</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>ICICIGI.NS</t>
-        </is>
-      </c>
-      <c r="D105" t="inlineStr"/>
+          <t>ONGC.NS</t>
+        </is>
+      </c>
+      <c r="D105" t="n">
+        <v>10.2</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Fin Services</t>
+          <t>Oil &amp; Gas</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Motilal Oswal Fin.</t>
+          <t>Gas Authority of India</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>MOTILALOFS.NS</t>
-        </is>
-      </c>
-      <c r="D106" t="inlineStr"/>
+          <t>GAIL.NS</t>
+        </is>
+      </c>
+      <c r="D106" t="n">
+        <v>3.8</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>FMCG</t>
+          <t>Oil &amp; Gas</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Dabur India</t>
+          <t>Reliance Industries</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>DABUR.NS</t>
-        </is>
-      </c>
-      <c r="D107" t="inlineStr"/>
+          <t>RELIANCE.NS</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
+        <v>45.2</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>FMCG</t>
+          <t>Pharma</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Varun Beverages</t>
+          <t>Sun Pharmaceutical</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>VARUNBEV.NS</t>
-        </is>
-      </c>
-      <c r="D108" t="inlineStr"/>
+          <t>SUNPHARMA.NS</t>
+        </is>
+      </c>
+      <c r="D108" t="n">
+        <v>18.5</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Infra</t>
+          <t>Pharma</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>IRB Infrastructure</t>
+          <t>Lupin Limited</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>IRB.NS</t>
-        </is>
-      </c>
-      <c r="D109" t="inlineStr"/>
+          <t>LUPIN.NS</t>
+        </is>
+      </c>
+      <c r="D109" t="n">
+        <v>14.2</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Infra</t>
+          <t>Pharma</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Adani Ports</t>
+          <t>Cipla</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>ADANIPORTS.NS</t>
-        </is>
-      </c>
-      <c r="D110" t="inlineStr"/>
+          <t>CIPLA.NS</t>
+        </is>
+      </c>
+      <c r="D110" t="n">
+        <v>12.8</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Pharma</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>L&amp;T Infotech</t>
+          <t>Dr. Reddy's Labs</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>LTIM.NS</t>
-        </is>
-      </c>
-      <c r="D111" t="inlineStr"/>
+          <t>DRREDDY.NS</t>
+        </is>
+      </c>
+      <c r="D111" t="n">
+        <v>11.5</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Pharma</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Dish TV India</t>
+          <t>Aurobindo Pharma</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>DISHTV.NS</t>
-        </is>
-      </c>
-      <c r="D112" t="inlineStr"/>
+          <t>AUROPHARMA.NS</t>
+        </is>
+      </c>
+      <c r="D112" t="n">
+        <v>9.699999999999999</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Metal</t>
+          <t>Pharma</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Hindustan Zinc</t>
+          <t>Divi's Laboratories</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>HINDZINC.NS</t>
-        </is>
-      </c>
-      <c r="D113" t="inlineStr"/>
+          <t>DIVISLAB.NS</t>
+        </is>
+      </c>
+      <c r="D113" t="n">
+        <v>8.300000000000001</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Oil &amp; Gas</t>
+          <t>Pharma</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Petronet LNG</t>
+          <t>IPCA Laboratories</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>PETRONET.NS</t>
-        </is>
-      </c>
-      <c r="D114" t="inlineStr"/>
+          <t>IPCALAB.NS</t>
+        </is>
+      </c>
+      <c r="D114" t="n">
+        <v>6.9</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -2686,33 +2646,37 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Biocon</t>
+          <t>Alembic Pharma</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>BIOCON.NS</t>
-        </is>
-      </c>
-      <c r="D115" t="inlineStr"/>
+          <t>APLLTD.NS</t>
+        </is>
+      </c>
+      <c r="D115" t="n">
+        <v>5.8</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Pharma</t>
+          <t>PSU Bank</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Glenmark Pharma</t>
+          <t>State Bank of India</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>GLENMARK.NS</t>
-        </is>
-      </c>
-      <c r="D116" t="inlineStr"/>
+          <t>SBIN.NS</t>
+        </is>
+      </c>
+      <c r="D116" t="n">
+        <v>38.2</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -2722,102 +2686,112 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Punjab National Bank</t>
+          <t>Central Bank</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>PNB.NS</t>
-        </is>
-      </c>
-      <c r="D117" t="inlineStr"/>
+          <t>CENTRALBK.NS</t>
+        </is>
+      </c>
+      <c r="D117" t="n">
+        <v>18.5</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Pvt Bank</t>
+          <t>PSU Bank</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Federal Bank</t>
+          <t>Bank of Baroda</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>FEDERALBNK.NS</t>
-        </is>
-      </c>
-      <c r="D118" t="inlineStr"/>
+          <t>BANKBARODA.NS</t>
+        </is>
+      </c>
+      <c r="D118" t="n">
+        <v>15.3</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Realty</t>
+          <t>PSU Bank</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Mahindra Lifespace</t>
+          <t>Indian Bank</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>MAHALXMI.NS</t>
-        </is>
-      </c>
-      <c r="D119" t="inlineStr"/>
+          <t>INDIANB.NS</t>
+        </is>
+      </c>
+      <c r="D119" t="n">
+        <v>12.1</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Nifty 50</t>
+          <t>PSU Bank</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Bharti Airtel</t>
+          <t>Canara Bank</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>BHARTIARTL.NS</t>
-        </is>
-      </c>
-      <c r="D120" t="inlineStr"/>
+          <t>CANBK.NS</t>
+        </is>
+      </c>
+      <c r="D120" t="n">
+        <v>9.800000000000001</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Auto</t>
+          <t>PSU Bank</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Apollo Tyres</t>
+          <t>Union Bank</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>APOLLOTYRE.NS</t>
-        </is>
-      </c>
-      <c r="D121" t="inlineStr"/>
+          <t>UNIONBANK.NS</t>
+        </is>
+      </c>
+      <c r="D121" t="n">
+        <v>4.2</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>FMCG</t>
+          <t>PSU Bank</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>United Spirits</t>
+          <t>Punjab National Bank</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>MCDOWELL-N.NS</t>
+          <t>PNB.NS</t>
         </is>
       </c>
       <c r="D122" t="inlineStr"/>
@@ -2825,182 +2799,202 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Infra</t>
+          <t>Pvt Bank</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>GMR Airports</t>
+          <t>HDFC Bank</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>GMRINFRA.NS</t>
-        </is>
-      </c>
-      <c r="D123" t="inlineStr"/>
+          <t>HDFCBANK.NS</t>
+        </is>
+      </c>
+      <c r="D123" t="n">
+        <v>28.5</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Pharma</t>
+          <t>Pvt Bank</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Torrent Pharma</t>
+          <t>ICICI Bank</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>TORNTPHARM.NS</t>
-        </is>
-      </c>
-      <c r="D124" t="inlineStr"/>
+          <t>ICICIBANK.NS</t>
+        </is>
+      </c>
+      <c r="D124" t="n">
+        <v>24.3</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>PSU Bank</t>
+          <t>Pvt Bank</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Bank of India</t>
+          <t>Axis Bank</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>BANKINDIA.NS</t>
-        </is>
-      </c>
-      <c r="D125" t="inlineStr"/>
+          <t>AXISBANK.NS</t>
+        </is>
+      </c>
+      <c r="D125" t="n">
+        <v>18.7</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Commodities</t>
+          <t>Pvt Bank</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>JSW Energy</t>
+          <t>Kotak Mahindra Bank</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>JSWENERGY.NS</t>
-        </is>
-      </c>
-      <c r="D126" t="inlineStr"/>
+          <t>KOTAKBANK.NS</t>
+        </is>
+      </c>
+      <c r="D126" t="n">
+        <v>15.2</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Defence</t>
+          <t>Pvt Bank</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Solar Industries</t>
+          <t>IDFC First Bank</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>SOLARA.NS</t>
-        </is>
-      </c>
-      <c r="D127" t="inlineStr"/>
+          <t>IDFCFIRSTB.NS</t>
+        </is>
+      </c>
+      <c r="D127" t="n">
+        <v>7.8</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>Fin Services</t>
+          <t>Pvt Bank</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>SBI Cards</t>
+          <t>IndusInd Bank</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>SBICARD.NS</t>
-        </is>
-      </c>
-      <c r="D128" t="inlineStr"/>
+          <t>INDUSINDBK.NS</t>
+        </is>
+      </c>
+      <c r="D128" t="n">
+        <v>4.2</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>FMCG</t>
+          <t>Realty</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Titan Company</t>
+          <t>DLF Limited</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>TITAN.NS</t>
-        </is>
-      </c>
-      <c r="D129" t="inlineStr"/>
+          <t>DLF.NS</t>
+        </is>
+      </c>
+      <c r="D129" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Realty</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>PVR Inox</t>
+          <t>Sunteck Realty</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>PVRINOX.NS</t>
-        </is>
-      </c>
-      <c r="D130" t="inlineStr"/>
+          <t>SUNTECK.NS</t>
+        </is>
+      </c>
+      <c r="D130" t="n">
+        <v>18.3</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>Metal</t>
+          <t>Realty</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Jindal Stainless</t>
+          <t>Oberoi Realty</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>JSL.NS</t>
-        </is>
-      </c>
-      <c r="D131" t="inlineStr"/>
+          <t>OBEROIRLTY.NS</t>
+        </is>
+      </c>
+      <c r="D131" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>Pvt Bank</t>
+          <t>Realty</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>Bandhan Bank</t>
+          <t>Prestige Estates</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>BANDHANBNK.NS</t>
-        </is>
-      </c>
-      <c r="D132" t="inlineStr"/>
+          <t>PRESTIGE.NS</t>
+        </is>
+      </c>
+      <c r="D132" t="n">
+        <v>11.8</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -3010,69 +3004,77 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>Sobha</t>
+          <t>Lodha Group</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>SOBHA.NS</t>
-        </is>
-      </c>
-      <c r="D133" t="inlineStr"/>
+          <t>LODHA.NS</t>
+        </is>
+      </c>
+      <c r="D133" t="n">
+        <v>10.2</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>Pharma</t>
+          <t>Realty</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>UPL Limited</t>
+          <t>Equinox India Developments (formerly Indiabulls)</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>UPL.NS</t>
-        </is>
-      </c>
-      <c r="D134" t="inlineStr"/>
+          <t>EQUINOX.NS</t>
+        </is>
+      </c>
+      <c r="D134" t="n">
+        <v>8.6</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>Auto</t>
+          <t>Realty</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>Escorts Kubota</t>
+          <t>Brigade Enterprises</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>ESCORTS.NS</t>
-        </is>
-      </c>
-      <c r="D135" t="inlineStr"/>
+          <t>BRIGADE.NS</t>
+        </is>
+      </c>
+      <c r="D135" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>Infra</t>
+          <t>Realty</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>Voltas</t>
+          <t>Godrej Properties</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>VOLTAS.NS</t>
-        </is>
-      </c>
-      <c r="D136" t="inlineStr"/>
+          <t>GODREJPROP.NS</t>
+        </is>
+      </c>
+      <c r="D136" t="n">
+        <v>6.7</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Sector-Company.xlsx (data file recompacted)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Sector-Company.xlsx
+++ b/Sector-Company.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Personal\Trading_Champion\Projects\Sector-rotation-v2\Sector-rotation-v2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B5E835B-8D8F-4D5E-AFBC-E467CC660FDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E1EFDAD-E566-4BB9-BED3-EB69D823D901}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="406" uniqueCount="286">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="403" uniqueCount="284">
   <si>
     <t>Sector</t>
   </si>
@@ -179,12 +179,6 @@
   </si>
   <si>
     <t>JINDALSTEL.NS</t>
-  </si>
-  <si>
-    <t>Manganese Ore India</t>
-  </si>
-  <si>
-    <t>MOIL.NS</t>
   </si>
   <si>
     <t>Vedanta</t>
@@ -1240,7 +1234,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D135"/>
+  <dimension ref="A1:D134"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="46.42578125" bestFit="1" customWidth="1"/>
@@ -1436,7 +1430,7 @@
         <v>4</v>
       </c>
       <c r="B15" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="C15" t="s">
         <v>31</v>
@@ -1581,26 +1575,23 @@
         <v>54</v>
       </c>
       <c r="D26">
-        <v>5.6</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>40</v>
+        <v>55</v>
       </c>
       <c r="B27" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C27" t="s">
-        <v>56</v>
-      </c>
-      <c r="D27">
-        <v>6.4</v>
+        <v>57</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B28" t="s">
         <v>58</v>
@@ -1611,7 +1602,7 @@
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B29" t="s">
         <v>60</v>
@@ -1622,7 +1613,7 @@
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B30" t="s">
         <v>62</v>
@@ -1633,7 +1624,7 @@
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B31" t="s">
         <v>64</v>
@@ -1644,7 +1635,7 @@
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B32" t="s">
         <v>66</v>
@@ -1655,7 +1646,7 @@
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B33" t="s">
         <v>68</v>
@@ -1666,7 +1657,7 @@
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B34" t="s">
         <v>70</v>
@@ -1677,7 +1668,7 @@
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B35" t="s">
         <v>72</v>
@@ -1688,18 +1679,21 @@
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>57</v>
+        <v>74</v>
       </c>
       <c r="B36" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C36" t="s">
-        <v>75</v>
+        <v>76</v>
+      </c>
+      <c r="D36">
+        <v>28.5</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B37" t="s">
         <v>77</v>
@@ -1708,12 +1702,12 @@
         <v>78</v>
       </c>
       <c r="D37">
-        <v>28.5</v>
+        <v>25.3</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B38" t="s">
         <v>79</v>
@@ -1722,12 +1716,12 @@
         <v>80</v>
       </c>
       <c r="D38">
-        <v>25.3</v>
+        <v>18.7</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B39" t="s">
         <v>81</v>
@@ -1736,26 +1730,26 @@
         <v>82</v>
       </c>
       <c r="D39">
-        <v>18.7</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="B40" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C40" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D40">
-        <v>5.2</v>
+        <v>35.200000000000003</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B41" t="s">
         <v>86</v>
@@ -1764,12 +1758,12 @@
         <v>87</v>
       </c>
       <c r="D41">
-        <v>35.200000000000003</v>
+        <v>18.899999999999999</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B42" t="s">
         <v>88</v>
@@ -1778,12 +1772,12 @@
         <v>89</v>
       </c>
       <c r="D42">
-        <v>18.899999999999999</v>
+        <v>12.3</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B43" t="s">
         <v>90</v>
@@ -1791,13 +1785,10 @@
       <c r="C43" t="s">
         <v>91</v>
       </c>
-      <c r="D43">
-        <v>12.3</v>
-      </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B44" t="s">
         <v>92</v>
@@ -1808,18 +1799,21 @@
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>85</v>
+        <v>94</v>
       </c>
       <c r="B45" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C45" t="s">
-        <v>95</v>
+        <v>96</v>
+      </c>
+      <c r="D45">
+        <v>15.4</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B46" t="s">
         <v>97</v>
@@ -1828,12 +1822,12 @@
         <v>98</v>
       </c>
       <c r="D46">
-        <v>15.4</v>
+        <v>8.1999999999999993</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B47" t="s">
         <v>99</v>
@@ -1842,12 +1836,12 @@
         <v>100</v>
       </c>
       <c r="D47">
-        <v>8.1999999999999993</v>
+        <v>6.85</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B48" t="s">
         <v>101</v>
@@ -1856,12 +1850,12 @@
         <v>102</v>
       </c>
       <c r="D48">
-        <v>6.85</v>
+        <v>6.32</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B49" t="s">
         <v>103</v>
@@ -1870,12 +1864,12 @@
         <v>104</v>
       </c>
       <c r="D49">
-        <v>6.32</v>
+        <v>5.68</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B50" t="s">
         <v>105</v>
@@ -1884,12 +1878,12 @@
         <v>106</v>
       </c>
       <c r="D50">
-        <v>5.68</v>
+        <v>5.37</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B51" t="s">
         <v>107</v>
@@ -1898,12 +1892,12 @@
         <v>108</v>
       </c>
       <c r="D51">
-        <v>5.37</v>
+        <v>4.74</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B52" t="s">
         <v>109</v>
@@ -1912,12 +1906,12 @@
         <v>110</v>
       </c>
       <c r="D52">
-        <v>4.74</v>
+        <v>4.2300000000000004</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B53" t="s">
         <v>111</v>
@@ -1926,12 +1920,12 @@
         <v>112</v>
       </c>
       <c r="D53">
-        <v>4.2300000000000004</v>
+        <v>3.66</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B54" t="s">
         <v>113</v>
@@ -1940,12 +1934,12 @@
         <v>114</v>
       </c>
       <c r="D54">
-        <v>3.66</v>
+        <v>3.34</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B55" t="s">
         <v>115</v>
@@ -1954,12 +1948,12 @@
         <v>116</v>
       </c>
       <c r="D55">
-        <v>3.34</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B56" t="s">
         <v>117</v>
@@ -1968,12 +1962,12 @@
         <v>118</v>
       </c>
       <c r="D56">
-        <v>1.9</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B57" t="s">
         <v>119</v>
@@ -1982,12 +1976,12 @@
         <v>120</v>
       </c>
       <c r="D57">
-        <v>1.3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B58" t="s">
         <v>121</v>
@@ -1995,13 +1989,10 @@
       <c r="C58" t="s">
         <v>122</v>
       </c>
-      <c r="D58">
-        <v>1</v>
-      </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B59" t="s">
         <v>123</v>
@@ -2012,7 +2003,7 @@
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B60" t="s">
         <v>125</v>
@@ -2023,18 +2014,21 @@
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>96</v>
+        <v>127</v>
       </c>
       <c r="B61" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C61" t="s">
-        <v>128</v>
+        <v>129</v>
+      </c>
+      <c r="D61">
+        <v>22.3</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B62" t="s">
         <v>130</v>
@@ -2043,12 +2037,12 @@
         <v>131</v>
       </c>
       <c r="D62">
-        <v>22.3</v>
+        <v>18.899999999999999</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B63" t="s">
         <v>132</v>
@@ -2057,12 +2051,12 @@
         <v>133</v>
       </c>
       <c r="D63">
-        <v>18.899999999999999</v>
+        <v>17.5</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B64" t="s">
         <v>134</v>
@@ -2071,12 +2065,12 @@
         <v>135</v>
       </c>
       <c r="D64">
-        <v>17.5</v>
+        <v>12.1</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B65" t="s">
         <v>136</v>
@@ -2085,12 +2079,12 @@
         <v>137</v>
       </c>
       <c r="D65">
-        <v>12.1</v>
+        <v>10.8</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B66" t="s">
         <v>138</v>
@@ -2099,12 +2093,12 @@
         <v>139</v>
       </c>
       <c r="D66">
-        <v>10.8</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B67" t="s">
         <v>140</v>
@@ -2113,12 +2107,12 @@
         <v>141</v>
       </c>
       <c r="D67">
-        <v>5.6</v>
+        <v>4.5999999999999996</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B68" t="s">
         <v>142</v>
@@ -2126,13 +2120,10 @@
       <c r="C68" t="s">
         <v>143</v>
       </c>
-      <c r="D68">
-        <v>4.5999999999999996</v>
-      </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B69" t="s">
         <v>144</v>
@@ -2143,7 +2134,7 @@
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B70" t="s">
         <v>146</v>
@@ -2154,7 +2145,7 @@
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B71" t="s">
         <v>148</v>
@@ -2165,18 +2156,21 @@
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>129</v>
+        <v>150</v>
       </c>
       <c r="B72" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C72" t="s">
-        <v>151</v>
+        <v>152</v>
+      </c>
+      <c r="D72">
+        <v>24.3</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="B73" t="s">
         <v>153</v>
@@ -2185,12 +2179,12 @@
         <v>154</v>
       </c>
       <c r="D73">
-        <v>24.3</v>
+        <v>15.8</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="B74" t="s">
         <v>155</v>
@@ -2199,12 +2193,12 @@
         <v>156</v>
       </c>
       <c r="D74">
-        <v>15.8</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="B75" t="s">
         <v>157</v>
@@ -2213,12 +2207,12 @@
         <v>158</v>
       </c>
       <c r="D75">
-        <v>12.5</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="B76" t="s">
         <v>159</v>
@@ -2226,13 +2220,10 @@
       <c r="C76" t="s">
         <v>160</v>
       </c>
-      <c r="D76">
-        <v>6.4</v>
-      </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="B77" t="s">
         <v>161</v>
@@ -2243,7 +2234,7 @@
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="B78" t="s">
         <v>163</v>
@@ -2254,7 +2245,7 @@
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="B79" t="s">
         <v>165</v>
@@ -2265,7 +2256,7 @@
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="B80" t="s">
         <v>167</v>
@@ -2276,7 +2267,7 @@
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="B81" t="s">
         <v>169</v>
@@ -2287,7 +2278,7 @@
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="B82" t="s">
         <v>171</v>
@@ -2298,7 +2289,7 @@
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="B83" t="s">
         <v>173</v>
@@ -2309,18 +2300,21 @@
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>152</v>
+        <v>175</v>
       </c>
       <c r="B84" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C84" t="s">
-        <v>176</v>
+        <v>177</v>
+      </c>
+      <c r="D84">
+        <v>20.5</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="B85" t="s">
         <v>178</v>
@@ -2329,12 +2323,12 @@
         <v>179</v>
       </c>
       <c r="D85">
-        <v>20.5</v>
+        <v>18.2</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="B86" t="s">
         <v>180</v>
@@ -2343,12 +2337,12 @@
         <v>181</v>
       </c>
       <c r="D86">
-        <v>18.2</v>
+        <v>12.1</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="B87" t="s">
         <v>182</v>
@@ -2357,12 +2351,12 @@
         <v>183</v>
       </c>
       <c r="D87">
-        <v>12.1</v>
+        <v>9.8000000000000007</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="B88" t="s">
         <v>184</v>
@@ -2371,12 +2365,12 @@
         <v>185</v>
       </c>
       <c r="D88">
-        <v>9.8000000000000007</v>
+        <v>7.3</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="B89" t="s">
         <v>186</v>
@@ -2385,12 +2379,12 @@
         <v>187</v>
       </c>
       <c r="D89">
-        <v>7.3</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="B90" t="s">
         <v>188</v>
@@ -2399,12 +2393,12 @@
         <v>189</v>
       </c>
       <c r="D90">
-        <v>6.4</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="B91" t="s">
         <v>190</v>
@@ -2413,12 +2407,12 @@
         <v>191</v>
       </c>
       <c r="D91">
-        <v>5.3</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="B92" t="s">
         <v>192</v>
@@ -2427,26 +2421,26 @@
         <v>193</v>
       </c>
       <c r="D92">
-        <v>5.2</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>177</v>
+        <v>194</v>
       </c>
       <c r="B93" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="C93" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="D93">
-        <v>4.0999999999999996</v>
+        <v>18.5</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="B94" t="s">
         <v>197</v>
@@ -2455,12 +2449,12 @@
         <v>198</v>
       </c>
       <c r="D94">
-        <v>18.5</v>
+        <v>12.8</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="B95" t="s">
         <v>199</v>
@@ -2469,12 +2463,12 @@
         <v>200</v>
       </c>
       <c r="D95">
-        <v>12.8</v>
+        <v>10.199999999999999</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="B96" t="s">
         <v>201</v>
@@ -2483,12 +2477,12 @@
         <v>202</v>
       </c>
       <c r="D96">
-        <v>10.199999999999999</v>
+        <v>8.9</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="B97" t="s">
         <v>203</v>
@@ -2496,24 +2490,24 @@
       <c r="C97" t="s">
         <v>204</v>
       </c>
-      <c r="D97">
-        <v>8.9</v>
-      </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>196</v>
+        <v>205</v>
       </c>
       <c r="B98" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="C98" t="s">
-        <v>206</v>
+        <v>207</v>
+      </c>
+      <c r="D98">
+        <v>27.7</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B99" t="s">
         <v>208</v>
@@ -2522,12 +2516,12 @@
         <v>209</v>
       </c>
       <c r="D99">
-        <v>27.7</v>
+        <v>17.899999999999999</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B100" t="s">
         <v>210</v>
@@ -2536,26 +2530,26 @@
         <v>211</v>
       </c>
       <c r="D100">
-        <v>17.899999999999999</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="B101" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C101" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="D101">
-        <v>5.7</v>
+        <v>22.3</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="B102" t="s">
         <v>215</v>
@@ -2564,12 +2558,12 @@
         <v>216</v>
       </c>
       <c r="D102">
-        <v>22.3</v>
+        <v>18.5</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="B103" t="s">
         <v>217</v>
@@ -2578,12 +2572,12 @@
         <v>218</v>
       </c>
       <c r="D103">
-        <v>18.5</v>
+        <v>10.199999999999999</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="B104" t="s">
         <v>219</v>
@@ -2592,40 +2586,40 @@
         <v>220</v>
       </c>
       <c r="D104">
-        <v>10.199999999999999</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="B105" t="s">
-        <v>221</v>
+        <v>84</v>
       </c>
       <c r="C105" t="s">
-        <v>222</v>
+        <v>85</v>
       </c>
       <c r="D105">
-        <v>3.8</v>
+        <v>45.2</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>214</v>
+        <v>221</v>
       </c>
       <c r="B106" t="s">
-        <v>86</v>
+        <v>222</v>
       </c>
       <c r="C106" t="s">
-        <v>87</v>
+        <v>223</v>
       </c>
       <c r="D106">
-        <v>45.2</v>
+        <v>18.5</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="B107" t="s">
         <v>224</v>
@@ -2634,12 +2628,12 @@
         <v>225</v>
       </c>
       <c r="D107">
-        <v>18.5</v>
+        <v>14.2</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="B108" t="s">
         <v>226</v>
@@ -2648,12 +2642,12 @@
         <v>227</v>
       </c>
       <c r="D108">
-        <v>14.2</v>
+        <v>12.8</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="B109" t="s">
         <v>228</v>
@@ -2662,12 +2656,12 @@
         <v>229</v>
       </c>
       <c r="D109">
-        <v>12.8</v>
+        <v>11.5</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="B110" t="s">
         <v>230</v>
@@ -2676,12 +2670,12 @@
         <v>231</v>
       </c>
       <c r="D110">
-        <v>11.5</v>
+        <v>9.6999999999999993</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="B111" t="s">
         <v>232</v>
@@ -2690,12 +2684,12 @@
         <v>233</v>
       </c>
       <c r="D111">
-        <v>9.6999999999999993</v>
+        <v>8.3000000000000007</v>
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="B112" t="s">
         <v>234</v>
@@ -2704,12 +2698,12 @@
         <v>235</v>
       </c>
       <c r="D112">
-        <v>8.3000000000000007</v>
+        <v>6.9</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="B113" t="s">
         <v>236</v>
@@ -2718,26 +2712,26 @@
         <v>237</v>
       </c>
       <c r="D113">
-        <v>6.9</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>223</v>
+        <v>238</v>
       </c>
       <c r="B114" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="C114" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="D114">
-        <v>5.8</v>
+        <v>38.200000000000003</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="B115" t="s">
         <v>241</v>
@@ -2746,12 +2740,12 @@
         <v>242</v>
       </c>
       <c r="D115">
-        <v>38.200000000000003</v>
+        <v>18.5</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="B116" t="s">
         <v>243</v>
@@ -2760,12 +2754,12 @@
         <v>244</v>
       </c>
       <c r="D116">
-        <v>18.5</v>
+        <v>15.3</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="B117" t="s">
         <v>245</v>
@@ -2774,12 +2768,12 @@
         <v>246</v>
       </c>
       <c r="D117">
-        <v>15.3</v>
+        <v>12.1</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="B118" t="s">
         <v>247</v>
@@ -2788,12 +2782,12 @@
         <v>248</v>
       </c>
       <c r="D118">
-        <v>12.1</v>
+        <v>9.8000000000000007</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="B119" t="s">
         <v>249</v>
@@ -2802,12 +2796,12 @@
         <v>250</v>
       </c>
       <c r="D119">
-        <v>9.8000000000000007</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="B120" t="s">
         <v>251</v>
@@ -2815,24 +2809,24 @@
       <c r="C120" t="s">
         <v>252</v>
       </c>
-      <c r="D120">
-        <v>4.2</v>
-      </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>240</v>
+        <v>253</v>
       </c>
       <c r="B121" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C121" t="s">
-        <v>254</v>
+        <v>255</v>
+      </c>
+      <c r="D121">
+        <v>28.5</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="B122" t="s">
         <v>256</v>
@@ -2841,12 +2835,12 @@
         <v>257</v>
       </c>
       <c r="D122">
-        <v>28.5</v>
+        <v>24.3</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="B123" t="s">
         <v>258</v>
@@ -2855,12 +2849,12 @@
         <v>259</v>
       </c>
       <c r="D123">
-        <v>24.3</v>
+        <v>18.7</v>
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="B124" t="s">
         <v>260</v>
@@ -2869,12 +2863,12 @@
         <v>261</v>
       </c>
       <c r="D124">
-        <v>18.7</v>
+        <v>15.2</v>
       </c>
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="B125" t="s">
         <v>262</v>
@@ -2883,12 +2877,12 @@
         <v>263</v>
       </c>
       <c r="D125">
-        <v>15.2</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="B126" t="s">
         <v>264</v>
@@ -2897,26 +2891,26 @@
         <v>265</v>
       </c>
       <c r="D126">
-        <v>7.8</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
-        <v>255</v>
+        <v>266</v>
       </c>
       <c r="B127" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C127" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D127">
-        <v>4.2</v>
+        <v>22.5</v>
       </c>
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="B128" t="s">
         <v>269</v>
@@ -2925,12 +2919,12 @@
         <v>270</v>
       </c>
       <c r="D128">
-        <v>22.5</v>
+        <v>18.3</v>
       </c>
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="B129" t="s">
         <v>271</v>
@@ -2939,12 +2933,12 @@
         <v>272</v>
       </c>
       <c r="D129">
-        <v>18.3</v>
+        <v>14</v>
       </c>
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="B130" t="s">
         <v>273</v>
@@ -2953,12 +2947,12 @@
         <v>274</v>
       </c>
       <c r="D130">
-        <v>14</v>
+        <v>11.8</v>
       </c>
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="B131" t="s">
         <v>275</v>
@@ -2967,12 +2961,12 @@
         <v>276</v>
       </c>
       <c r="D131">
-        <v>11.8</v>
+        <v>10.199999999999999</v>
       </c>
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="B132" t="s">
         <v>277</v>
@@ -2981,12 +2975,12 @@
         <v>278</v>
       </c>
       <c r="D132">
-        <v>10.199999999999999</v>
+        <v>8.6</v>
       </c>
     </row>
     <row r="133" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="B133" t="s">
         <v>279</v>
@@ -2995,12 +2989,12 @@
         <v>280</v>
       </c>
       <c r="D133">
-        <v>8.6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="134" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="B134" t="s">
         <v>281</v>
@@ -3009,20 +3003,6 @@
         <v>282</v>
       </c>
       <c r="D134">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="135" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A135" t="s">
-        <v>268</v>
-      </c>
-      <c r="B135" t="s">
-        <v>283</v>
-      </c>
-      <c r="C135" t="s">
-        <v>284</v>
-      </c>
-      <c r="D135">
         <v>6.7</v>
       </c>
     </row>

</xml_diff>